<commit_message>
update to add outdated flag
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -41213,7 +41213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W8"/>
+  <dimension ref="A1:W14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41875,6 +41875,468 @@
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2025021070</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Greaves</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-129</v>
+      </c>
+      <c r="G9" t="n">
+        <v>105</v>
+      </c>
+      <c r="H9" t="n">
+        <v>8482982</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>CBJ</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>CAR</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>1</v>
+      </c>
+      <c r="L9" t="n">
+        <v>25.60000038146973</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.317453145980835</v>
+      </c>
+      <c r="N9" t="n">
+        <v>36.50936889648438</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>65-70%</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>UNDER</t>
+        </is>
+      </c>
+      <c r="Q9" t="n">
+        <v>0.19474196434021</v>
+      </c>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2025021072</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Gustavsson</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-112</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-110</v>
+      </c>
+      <c r="H10" t="n">
+        <v>8479406</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>MIN</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>CHI</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>23.20000076293945</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.6459309458732605</v>
+      </c>
+      <c r="N10" t="n">
+        <v>29.18618965148926</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>60-65%</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>0.1176290512084961</v>
+      </c>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2025021073</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Ingram</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-110</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-112</v>
+      </c>
+      <c r="H11" t="n">
+        <v>8478971</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>EDM</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>SJS</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" t="n">
+        <v>21.39999961853027</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.4727703332901001</v>
+      </c>
+      <c r="N11" t="n">
+        <v>5.44593334197998</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>50-55%</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q11" t="n">
+        <v>-0.001072227954864502</v>
+      </c>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>2025021070</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Bussi</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-120</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-103</v>
+      </c>
+      <c r="H12" t="n">
+        <v>8483548</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>CAR</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>CBJ</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
+        <v>23.10000038146973</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.6182592511177063</v>
+      </c>
+      <c r="N12" t="n">
+        <v>23.6518497467041</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>60-65%</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q12" t="n">
+        <v>0.07280468940734863</v>
+      </c>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2025021068</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Woll</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-130</v>
+      </c>
+      <c r="G13" t="n">
+        <v>106</v>
+      </c>
+      <c r="H13" t="n">
+        <v>8479361</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>NYI</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" t="n">
+        <v>26.70000076293945</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.5444204807281494</v>
+      </c>
+      <c r="N13" t="n">
+        <v>8.884096145629883</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>50-55%</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q13" t="n">
+        <v>-0.02079689502716064</v>
+      </c>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr"/>
+      <c r="W13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2025021071</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Saros</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-120</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-104</v>
+      </c>
+      <c r="H14" t="n">
+        <v>8477424</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>NSH</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>WPG</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
+        <v>24.60000038146973</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0.525579571723938</v>
+      </c>
+      <c r="N14" t="n">
+        <v>5.115914344787598</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>50-55%</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q14" t="n">
+        <v>-0.01987498998641968</v>
+      </c>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update betting_tracker with latest predictions
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -45560,7 +45560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W19"/>
+  <dimension ref="A1:W25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -47069,6 +47069,468 @@
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>2025021089</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Ingram</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="F20" t="n">
+        <v>100</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-122</v>
+      </c>
+      <c r="H20" t="n">
+        <v>8478971</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>EDM</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>FLA</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>1</v>
+      </c>
+      <c r="L20" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0.3241397440433502</v>
+      </c>
+      <c r="N20" t="n">
+        <v>35.17205119132996</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>65-70%</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>UNDER</t>
+        </is>
+      </c>
+      <c r="Q20" t="n">
+        <v>0.1263107064071002</v>
+      </c>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2025021093</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Kuemper</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="F21" t="n">
+        <v>-117</v>
+      </c>
+      <c r="G21" t="n">
+        <v>-106</v>
+      </c>
+      <c r="H21" t="n">
+        <v>8475311</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>LAK</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
+        <v>1</v>
+      </c>
+      <c r="L21" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0.5161674022674561</v>
+      </c>
+      <c r="N21" t="n">
+        <v>3.233480453491211</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>50-55%</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q21" t="n">
+        <v>-0.02300310464498634</v>
+      </c>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>2025021092</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Nedeljkovic</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="F22" t="n">
+        <v>-103</v>
+      </c>
+      <c r="G22" t="n">
+        <v>-121</v>
+      </c>
+      <c r="H22" t="n">
+        <v>8477968</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>SJS</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>BUF</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
+        <v>1</v>
+      </c>
+      <c r="L22" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0.3311481177806854</v>
+      </c>
+      <c r="N22" t="n">
+        <v>33.77037644386292</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>65-70%</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>UNDER</t>
+        </is>
+      </c>
+      <c r="Q22" t="n">
+        <v>0.12134057000212</v>
+      </c>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="inlineStr"/>
+      <c r="W22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>2025021092</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Lyon</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="F23" t="n">
+        <v>-108</v>
+      </c>
+      <c r="G23" t="n">
+        <v>-114</v>
+      </c>
+      <c r="H23" t="n">
+        <v>8479312</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>BUF</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>SJS</t>
+        </is>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0.3103089332580566</v>
+      </c>
+      <c r="N23" t="n">
+        <v>37.93821334838867</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>65-70%</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>UNDER</t>
+        </is>
+      </c>
+      <c r="Q23" t="n">
+        <v>0.1569807863681116</v>
+      </c>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr"/>
+      <c r="W23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>2025021090</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Lankinen</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="F24" t="n">
+        <v>-102</v>
+      </c>
+      <c r="G24" t="n">
+        <v>-122</v>
+      </c>
+      <c r="H24" t="n">
+        <v>8480947</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>VAN</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>TBL</t>
+        </is>
+      </c>
+      <c r="K24" t="n">
+        <v>1</v>
+      </c>
+      <c r="L24" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0.3021916151046753</v>
+      </c>
+      <c r="N24" t="n">
+        <v>39.56167697906494</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>65-70%</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>UNDER</t>
+        </is>
+      </c>
+      <c r="Q24" t="n">
+        <v>0.1482588353457751</v>
+      </c>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>2025021093</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Ersson</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F25" t="n">
+        <v>-104</v>
+      </c>
+      <c r="G25" t="n">
+        <v>-118</v>
+      </c>
+      <c r="H25" t="n">
+        <v>8481035</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>LAK</t>
+        </is>
+      </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="M25" t="n">
+        <v>0.3202995359897614</v>
+      </c>
+      <c r="N25" t="n">
+        <v>35.94009280204773</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>65-70%</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>UNDER</t>
+        </is>
+      </c>
+      <c r="Q25" t="n">
+        <v>0.1384160603405139</v>
+      </c>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr"/>
+      <c r="W25" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update betting_tracker with latest predictions (#12)
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -1,41 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-20" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-19" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-18" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-17" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-16" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-15" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-14" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-13" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-12" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-11" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-10" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-09" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-07" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-06" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-05" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-04" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-03" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-02" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-01" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-02-28" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-02-27" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-02-26" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-02-25" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-02-05" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-02-04" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-02-03" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-02-02" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-02-01" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Settings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2026-03-20" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2026-03-19" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="2026-03-18" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="2026-03-17" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="2026-03-16" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="2026-03-15" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="2026-03-14" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="2026-03-13" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="2026-03-12" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="2026-03-11" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="2026-03-10" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="2026-03-09" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="2026-03-07" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="2026-03-06" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="2026-03-05" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="2026-03-04" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="2026-03-03" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="2026-03-02" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="2026-03-01" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="2026-02-28" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="2026-02-27" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="2026-02-26" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="2026-02-25" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="2026-02-05" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="2026-02-04" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="2026-02-03" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="2026-02-02" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="2026-02-01" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -45796,7 +45796,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W7"/>
+  <dimension ref="A1:W15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -46038,17 +46038,17 @@
         <v>1</v>
       </c>
       <c r="L3" t="n">
-        <v>28.20000076293945</v>
+        <v>28</v>
       </c>
       <c r="M3" t="n">
-        <v>0.4487713277339935</v>
+        <v>0.3903127610683441</v>
       </c>
       <c r="N3" t="n">
-        <v>10.24573421478271</v>
+        <v>21.93744778633118</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>55-60%</t>
+          <t>60-65%</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -46057,7 +46057,7 @@
         </is>
       </c>
       <c r="Q3" t="n">
-        <v>0.02741909027099609</v>
+        <v>0.08587771512213205</v>
       </c>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
@@ -46115,13 +46115,13 @@
         <v>1</v>
       </c>
       <c r="L4" t="n">
-        <v>25.70000076293945</v>
+        <v>25.4</v>
       </c>
       <c r="M4" t="n">
-        <v>0.5455245971679688</v>
+        <v>0.4855647087097168</v>
       </c>
       <c r="N4" t="n">
-        <v>9.10491943359375</v>
+        <v>2.887058258056641</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -46134,7 +46134,7 @@
         </is>
       </c>
       <c r="Q4" t="n">
-        <v>-0.008046805858612061</v>
+        <v>0.01692285347933792</v>
       </c>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr">
@@ -46192,17 +46192,17 @@
         <v>1</v>
       </c>
       <c r="L5" t="n">
-        <v>30</v>
+        <v>29.7</v>
       </c>
       <c r="M5" t="n">
-        <v>0.3905491828918457</v>
+        <v>0.3350647687911987</v>
       </c>
       <c r="N5" t="n">
-        <v>21.89016342163086</v>
+        <v>32.98704624176025</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>60-65%</t>
+          <t>65-70%</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -46211,7 +46211,7 @@
         </is>
       </c>
       <c r="Q5" t="n">
-        <v>0.06399625539779663</v>
+        <v>0.1194806857542559</v>
       </c>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr">
@@ -46269,13 +46269,13 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>23.60000038146973</v>
+        <v>23.3</v>
       </c>
       <c r="M6" t="n">
-        <v>0.516499936580658</v>
+        <v>0.4565255641937256</v>
       </c>
       <c r="N6" t="n">
-        <v>3.299987316131592</v>
+        <v>8.694887161254883</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -46288,7 +46288,7 @@
         </is>
       </c>
       <c r="Q6" t="n">
-        <v>-0.01649993658065796</v>
+        <v>0.04347443580627441</v>
       </c>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr">
@@ -46346,17 +46346,17 @@
         <v>1</v>
       </c>
       <c r="L7" t="n">
-        <v>25.70000076293945</v>
+        <v>25.4</v>
       </c>
       <c r="M7" t="n">
-        <v>0.3404632806777954</v>
+        <v>0.28872349858284</v>
       </c>
       <c r="N7" t="n">
-        <v>31.90734481811523</v>
+        <v>42.25530028343201</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>65-70%</t>
+          <t>70-75%</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -46365,7 +46365,7 @@
         </is>
       </c>
       <c r="Q7" t="n">
-        <v>0.1246529817581177</v>
+        <v>0.1763927804869275</v>
       </c>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr">
@@ -46377,6 +46377,622 @@
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2025021095</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Thompson</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-124</v>
+      </c>
+      <c r="G8" t="n">
+        <v>101</v>
+      </c>
+      <c r="H8" t="n">
+        <v>8480313</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>WSH</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>NJD</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.4855647087097168</v>
+      </c>
+      <c r="N8" t="n">
+        <v>2.887058258056641</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>50-55%</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
+        <v>0.01692285347933792</v>
+      </c>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2025021095</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Allen</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-122</v>
+      </c>
+      <c r="G9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H9" t="n">
+        <v>8474596</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>NJD</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>WSH</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.4565255641937256</v>
+      </c>
+      <c r="N9" t="n">
+        <v>8.694887161254883</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>50-55%</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q9" t="n">
+        <v>0.04347443580627441</v>
+      </c>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2025021094</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Bussi</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-121</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-102</v>
+      </c>
+      <c r="H10" t="n">
+        <v>8483548</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>CAR</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.4673799276351929</v>
+      </c>
+      <c r="N10" t="n">
+        <v>6.524014472961426</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>50-55%</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>0.02766957731530217</v>
+      </c>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2025021094</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Woll</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-104</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-120</v>
+      </c>
+      <c r="H11" t="n">
+        <v>8479361</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>CAR</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.3350647687911987</v>
+      </c>
+      <c r="N11" t="n">
+        <v>32.98704624176025</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>65-70%</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q11" t="n">
+        <v>0.1194806857542559</v>
+      </c>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>2025021096</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Blackwood</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-115</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-107</v>
+      </c>
+      <c r="H12" t="n">
+        <v>8478406</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>CHI</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.5026932954788208</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0.5386590957641602</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>50-55%</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q12" t="n">
+        <v>-0.01960150803920724</v>
+      </c>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2025021096</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Soderblom</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-112</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-110</v>
+      </c>
+      <c r="H13" t="n">
+        <v>8482821</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>CHI</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" t="n">
+        <v>28</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.3903127610683441</v>
+      </c>
+      <c r="N13" t="n">
+        <v>21.93744778633118</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>60-65%</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q13" t="n">
+        <v>0.08587771512213205</v>
+      </c>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr"/>
+      <c r="W13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2025021097</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Wolf</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-107</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-115</v>
+      </c>
+      <c r="H14" t="n">
+        <v>8481692</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>CGY</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>FLA</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L14" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0.28872349858284</v>
+      </c>
+      <c r="N14" t="n">
+        <v>42.25530028343201</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>70-75%</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>UNDER</t>
+        </is>
+      </c>
+      <c r="Q14" t="n">
+        <v>0.1763927804869275</v>
+      </c>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2025021098</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Vejmelka</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-105</v>
+      </c>
+      <c r="G15" t="n">
+        <v>-118</v>
+      </c>
+      <c r="H15" t="n">
+        <v>8478872</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>UTA</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>ANA</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>1</v>
+      </c>
+      <c r="L15" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0.5190231800079346</v>
+      </c>
+      <c r="N15" t="n">
+        <v>3.804636001586914</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>50-55%</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q15" t="n">
+        <v>0.006828058056715047</v>
+      </c>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr"/>
+      <c r="W15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update betting_tracker with latest predictions (#14)
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -45796,7 +45796,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W15"/>
+  <dimension ref="A1:W21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -46993,6 +46993,468 @@
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2025021095</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Allen</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-125</v>
+      </c>
+      <c r="G16" t="n">
+        <v>103</v>
+      </c>
+      <c r="H16" t="n">
+        <v>8474596</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>NJD</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>WSH</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0.4565255641937256</v>
+      </c>
+      <c r="N16" t="n">
+        <v>8.694887161254883</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>50-55%</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q16" t="n">
+        <v>0.05086359836785076</v>
+      </c>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>2025021095</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Thompson</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="F17" t="n">
+        <v>-125</v>
+      </c>
+      <c r="G17" t="n">
+        <v>103</v>
+      </c>
+      <c r="H17" t="n">
+        <v>8480313</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>WSH</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>NJD</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>1</v>
+      </c>
+      <c r="L17" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0.4855647087097168</v>
+      </c>
+      <c r="N17" t="n">
+        <v>2.887058258056641</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>50-55%</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q17" t="n">
+        <v>0.02182445385185955</v>
+      </c>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr"/>
+      <c r="W17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>2025021094</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Bussi</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="F18" t="n">
+        <v>-125</v>
+      </c>
+      <c r="G18" t="n">
+        <v>103</v>
+      </c>
+      <c r="H18" t="n">
+        <v>8483548</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>CAR</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0.4673799276351929</v>
+      </c>
+      <c r="N18" t="n">
+        <v>6.524014472961426</v>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>50-55%</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q18" t="n">
+        <v>0.04000923492638347</v>
+      </c>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr"/>
+      <c r="W18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>2025021097</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Tarasov</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F19" t="n">
+        <v>-104</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-118</v>
+      </c>
+      <c r="H19" t="n">
+        <v>8480193</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>FLA</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>CGY</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0.5870197415351868</v>
+      </c>
+      <c r="N19" t="n">
+        <v>17.40394830703735</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>55-60%</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q19" t="n">
+        <v>0.07721581996655935</v>
+      </c>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr"/>
+      <c r="W19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>2025021097</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Wolf</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="F20" t="n">
+        <v>-103</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-120</v>
+      </c>
+      <c r="H20" t="n">
+        <v>8481692</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>CGY</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>FLA</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>1</v>
+      </c>
+      <c r="L20" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0.28872349858284</v>
+      </c>
+      <c r="N20" t="n">
+        <v>42.25530028343201</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>70-75%</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>UNDER</t>
+        </is>
+      </c>
+      <c r="Q20" t="n">
+        <v>0.1658219559626146</v>
+      </c>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2025021098</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Dostal</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="F21" t="n">
+        <v>-122</v>
+      </c>
+      <c r="G21" t="n">
+        <v>-102</v>
+      </c>
+      <c r="H21" t="n">
+        <v>8480843</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>ANA</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>UTA</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0.2419283390045166</v>
+      </c>
+      <c r="N21" t="n">
+        <v>51.61433219909668</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>75%+</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>UNDER</t>
+        </is>
+      </c>
+      <c r="Q21" t="n">
+        <v>0.2531211659459784</v>
+      </c>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update betting_tracker with latest predictions (#17)
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -1,45 +1,45 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-24" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-23" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-22" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-21" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-20" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-19" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-18" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-17" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-16" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-15" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-14" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-13" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-12" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-11" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-10" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-09" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-07" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-06" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-05" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-04" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-03" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-02" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-01" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-02-28" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-02-27" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-02-26" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-02-25" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-02-05" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-02-04" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-02-03" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-02-02" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-02-01" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Settings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2026-03-24" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2026-03-23" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="2026-03-22" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="2026-03-21" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="2026-03-20" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="2026-03-19" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="2026-03-18" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="2026-03-17" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="2026-03-16" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="2026-03-15" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="2026-03-14" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="2026-03-13" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="2026-03-12" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="2026-03-11" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="2026-03-10" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="2026-03-09" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="2026-03-07" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="2026-03-06" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="2026-03-05" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="2026-03-04" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="2026-03-03" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="2026-03-02" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="2026-03-01" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="2026-02-28" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="2026-02-27" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="2026-02-26" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="2026-02-25" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="2026-02-05" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="2026-02-04" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="2026-02-03" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="2026-02-02" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="2026-02-01" sheetId="34" state="visible" r:id="rId34"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -40289,7 +40289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W39"/>
+  <dimension ref="A1:W69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40533,26 +40533,26 @@
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>23.10000038146973</v>
+        <v>22.8</v>
       </c>
       <c r="M3" t="n">
-        <v>0.4273654520511627</v>
+        <v>0.3698245584964752</v>
       </c>
       <c r="N3" t="n">
-        <v>14.52690982818604</v>
+        <v>26.03508830070496</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>55-60%</t>
+          <t>60-65%</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>NO BET</t>
+          <t>UNDER</t>
         </is>
       </c>
       <c r="Q3" t="n">
-        <v>0.07263457775115967</v>
+        <v>0.1301754415035248</v>
       </c>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
@@ -40610,17 +40610,17 @@
         <v>1</v>
       </c>
       <c r="L4" t="n">
-        <v>27.39999961853027</v>
+        <v>27.1</v>
       </c>
       <c r="M4" t="n">
-        <v>0.480671614408493</v>
+        <v>0.4212331175804138</v>
       </c>
       <c r="N4" t="n">
-        <v>3.865677118301392</v>
+        <v>15.75337648391724</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>50-55%</t>
+          <t>55-60%</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -40629,7 +40629,7 @@
         </is>
       </c>
       <c r="Q4" t="n">
-        <v>-0.0111880898475647</v>
+        <v>0.04825045049470356</v>
       </c>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr">
@@ -40687,26 +40687,26 @@
         <v>1</v>
       </c>
       <c r="L5" t="n">
-        <v>23.89999961853027</v>
+        <v>23.6</v>
       </c>
       <c r="M5" t="n">
-        <v>0.3835527896881104</v>
+        <v>0.3285265266895294</v>
       </c>
       <c r="N5" t="n">
-        <v>23.28944206237793</v>
+        <v>34.29469466209412</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>60-65%</t>
+          <t>65-70%</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>NO BET</t>
+          <t>UNDER</t>
         </is>
       </c>
       <c r="Q5" t="n">
-        <v>0.09263765811920166</v>
+        <v>0.1476639495009467</v>
       </c>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr">
@@ -40841,26 +40841,26 @@
         <v>1</v>
       </c>
       <c r="L7" t="n">
-        <v>22.60000038146973</v>
+        <v>22.1</v>
       </c>
       <c r="M7" t="n">
-        <v>0.7181222438812256</v>
+        <v>0.6140996217727661</v>
       </c>
       <c r="N7" t="n">
-        <v>43.62445068359375</v>
+        <v>22.81992435455322</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>70-75%</t>
+          <t>60-65%</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>OVER</t>
+          <t>NO BET</t>
         </is>
       </c>
       <c r="Q7" t="n">
-        <v>0.1898203492164612</v>
+        <v>0.08579773498031329</v>
       </c>
       <c r="R7" t="n">
         <v>1</v>
@@ -40920,17 +40920,17 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>25.89999961853027</v>
+        <v>25.6</v>
       </c>
       <c r="M8" t="n">
-        <v>0.5817586779594421</v>
+        <v>0.5223939418792725</v>
       </c>
       <c r="N8" t="n">
-        <v>16.35173606872559</v>
+        <v>4.478788375854492</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>55-60%</t>
+          <t>50-55%</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -40939,7 +40939,7 @@
         </is>
       </c>
       <c r="Q8" t="n">
-        <v>0.02818727493286133</v>
+        <v>-0.01990637969021775</v>
       </c>
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr">
@@ -41153,17 +41153,17 @@
         <v>1</v>
       </c>
       <c r="L11" t="n">
-        <v>22.20000076293945</v>
+        <v>21.9</v>
       </c>
       <c r="M11" t="n">
-        <v>0.636540412902832</v>
+        <v>0.579328715801239</v>
       </c>
       <c r="N11" t="n">
-        <v>27.30808258056641</v>
+        <v>15.8657431602478</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>60-65%</t>
+          <t>55-60%</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -41172,7 +41172,7 @@
         </is>
       </c>
       <c r="Q11" t="n">
-        <v>0.1173096299171448</v>
+        <v>0.06009794657046974</v>
       </c>
       <c r="R11" t="n">
         <v>1</v>
@@ -41232,17 +41232,17 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>26.10000038146973</v>
+        <v>25.8</v>
       </c>
       <c r="M12" t="n">
-        <v>0.4174536764621735</v>
+        <v>0.3604073524475098</v>
       </c>
       <c r="N12" t="n">
-        <v>16.50926399230957</v>
+        <v>27.91852951049805</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>55-60%</t>
+          <t>60-65%</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -41251,7 +41251,7 @@
         </is>
       </c>
       <c r="Q12" t="n">
-        <v>0.04983609914779663</v>
+        <v>0.1068823671786585</v>
       </c>
       <c r="R12" t="n">
         <v>1</v>
@@ -41311,13 +41311,13 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>27.70000076293945</v>
+        <v>27.4</v>
       </c>
       <c r="M13" t="n">
-        <v>0.5375425219535828</v>
+        <v>0.4775381088256836</v>
       </c>
       <c r="N13" t="n">
-        <v>7.508504390716553</v>
+        <v>4.492378234863281</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -41330,7 +41330,7 @@
         </is>
       </c>
       <c r="Q13" t="n">
-        <v>0.02297943830490112</v>
+        <v>-0.01670861573812599</v>
       </c>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr">
@@ -41388,17 +41388,17 @@
         <v>1</v>
       </c>
       <c r="L14" t="n">
-        <v>23.5</v>
+        <v>23.2</v>
       </c>
       <c r="M14" t="n">
-        <v>0.4914213716983795</v>
+        <v>0.4317587614059448</v>
       </c>
       <c r="N14" t="n">
-        <v>1.715725660324097</v>
+        <v>13.64824771881104</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>50-55%</t>
+          <t>55-60%</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -41407,7 +41407,7 @@
         </is>
       </c>
       <c r="Q14" t="n">
-        <v>-0.01972323656082153</v>
+        <v>0.03993935180160235</v>
       </c>
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr">
@@ -41465,17 +41465,17 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>25.39999961853027</v>
+        <v>25.2</v>
       </c>
       <c r="M15" t="n">
-        <v>0.2753289639949799</v>
+        <v>0.2300351709127426</v>
       </c>
       <c r="N15" t="n">
-        <v>44.93420791625977</v>
+        <v>53.99296581745148</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>70-75%</t>
+          <t>75%+</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -41484,7 +41484,7 @@
         </is>
       </c>
       <c r="Q15" t="n">
-        <v>0.1710996031761169</v>
+        <v>0.2163934005158288</v>
       </c>
       <c r="R15" t="n">
         <v>2</v>
@@ -41702,13 +41702,13 @@
         <v>1</v>
       </c>
       <c r="L18" t="n">
-        <v>24.70000076293945</v>
+        <v>24.3</v>
       </c>
       <c r="M18" t="n">
-        <v>0.5300005674362183</v>
+        <v>0.4699823558330536</v>
       </c>
       <c r="N18" t="n">
-        <v>6.000113487243652</v>
+        <v>6.003528833389282</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -41721,7 +41721,7 @@
         </is>
       </c>
       <c r="Q18" t="n">
-        <v>0.01543748378753662</v>
+        <v>-0.009152862745495982</v>
       </c>
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr">
@@ -41858,26 +41858,26 @@
         <v>1</v>
       </c>
       <c r="L20" t="n">
-        <v>24.79999923706055</v>
+        <v>24.5</v>
       </c>
       <c r="M20" t="n">
-        <v>0.3616737723350525</v>
+        <v>0.3082170188426971</v>
       </c>
       <c r="N20" t="n">
-        <v>27.66524505615234</v>
+        <v>38.35659623146057</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>60-65%</t>
+          <t>65-70%</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>NO BET</t>
+          <t>UNDER</t>
         </is>
       </c>
       <c r="Q20" t="n">
-        <v>0.09287166595458984</v>
+        <v>0.1463284357027574</v>
       </c>
       <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr">
@@ -41935,26 +41935,26 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>23.29999923706055</v>
+        <v>23</v>
       </c>
       <c r="M21" t="n">
-        <v>0.6518069505691528</v>
+        <v>0.595471203327179</v>
       </c>
       <c r="N21" t="n">
-        <v>30.36138916015625</v>
+        <v>19.09424066543579</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>65-70%</t>
+          <t>55-60%</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>OVER</t>
+          <t>NO BET</t>
         </is>
       </c>
       <c r="Q21" t="n">
-        <v>0.1567574441432953</v>
+        <v>0.1004216983766839</v>
       </c>
       <c r="R21" t="n">
         <v>1</v>
@@ -42014,13 +42014,13 @@
         <v>1</v>
       </c>
       <c r="L22" t="n">
-        <v>23.79999923706055</v>
+        <v>25.1</v>
       </c>
       <c r="M22" t="n">
-        <v>0.3560058176517487</v>
+        <v>0.6251416206359863</v>
       </c>
       <c r="N22" t="n">
-        <v>28.79883575439453</v>
+        <v>25.02832412719727</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -42033,7 +42033,7 @@
         </is>
       </c>
       <c r="Q22" t="n">
-        <v>0.1091104745864868</v>
+        <v>0.1082334080755999</v>
       </c>
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr">
@@ -42091,13 +42091,13 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>22.89999961853027</v>
+        <v>24.2</v>
       </c>
       <c r="M23" t="n">
-        <v>0.3718112707138062</v>
+        <v>0.6457219123840332</v>
       </c>
       <c r="N23" t="n">
-        <v>25.63774490356445</v>
+        <v>29.14438247680664</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -42106,11 +42106,11 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>NO BET</t>
+          <t>OVER</t>
         </is>
       </c>
       <c r="Q23" t="n">
-        <v>0.06297135353088379</v>
+        <v>0.1626301249444197</v>
       </c>
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr">
@@ -42245,17 +42245,17 @@
         <v>1</v>
       </c>
       <c r="L25" t="n">
-        <v>24.39999961853027</v>
+        <v>24.2</v>
       </c>
       <c r="M25" t="n">
-        <v>0.2844393849372864</v>
+        <v>0.2381392866373062</v>
       </c>
       <c r="N25" t="n">
-        <v>43.11212158203125</v>
+        <v>52.37214267253876</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>70-75%</t>
+          <t>75%+</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
@@ -42264,7 +42264,7 @@
         </is>
       </c>
       <c r="Q25" t="n">
-        <v>0.1660110950469971</v>
+        <v>0.2123111638131442</v>
       </c>
       <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr">
@@ -42322,17 +42322,17 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>25.39999961853027</v>
+        <v>25.1</v>
       </c>
       <c r="M26" t="n">
-        <v>0.4814599752426147</v>
+        <v>0.4220030903816223</v>
       </c>
       <c r="N26" t="n">
-        <v>3.708004951477051</v>
+        <v>15.59938192367554</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>50-55%</t>
+          <t>55-60%</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -42341,7 +42341,7 @@
         </is>
       </c>
       <c r="Q26" t="n">
-        <v>-0.01634371280670166</v>
+        <v>0.04311318868814518</v>
       </c>
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr">
@@ -42399,17 +42399,17 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>22.10000038146973</v>
+        <v>21.8</v>
       </c>
       <c r="M27" t="n">
-        <v>0.6146973967552185</v>
+        <v>0.5564432144165039</v>
       </c>
       <c r="N27" t="n">
-        <v>22.93947982788086</v>
+        <v>11.28864288330078</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>60-65%</t>
+          <t>55-60%</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -42418,7 +42418,7 @@
         </is>
       </c>
       <c r="Q27" t="n">
-        <v>0.0931662917137146</v>
+        <v>0.03491211393803506</v>
       </c>
       <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr">
@@ -42476,17 +42476,17 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>23.29999923706055</v>
+        <v>23</v>
       </c>
       <c r="M28" t="n">
-        <v>0.4689461886882782</v>
+        <v>0.409813404083252</v>
       </c>
       <c r="N28" t="n">
-        <v>6.210762023925781</v>
+        <v>18.03731918334961</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>50-55%</t>
+          <t>55-60%</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
@@ -42495,7 +42495,7 @@
         </is>
       </c>
       <c r="Q28" t="n">
-        <v>-0.0225176215171814</v>
+        <v>0.03661516734531944</v>
       </c>
       <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr">
@@ -42553,13 +42553,13 @@
         <v>1</v>
       </c>
       <c r="L29" t="n">
-        <v>24.60000038146973</v>
+        <v>24.3</v>
       </c>
       <c r="M29" t="n">
-        <v>0.5152634382247925</v>
+        <v>0.4552974998950958</v>
       </c>
       <c r="N29" t="n">
-        <v>3.052687644958496</v>
+        <v>8.940500020980835</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -42572,7 +42572,7 @@
         </is>
       </c>
       <c r="Q29" t="n">
-        <v>-0.001644790172576904</v>
+        <v>0.01199221973107245</v>
       </c>
       <c r="R29" t="inlineStr"/>
       <c r="S29" t="inlineStr">
@@ -42630,13 +42630,13 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>23.70000076293945</v>
+        <v>23.4</v>
       </c>
       <c r="M30" t="n">
-        <v>0.5419632196426392</v>
+        <v>0.4819795787334442</v>
       </c>
       <c r="N30" t="n">
-        <v>8.392643928527832</v>
+        <v>3.604084253311157</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -42649,7 +42649,7 @@
         </is>
       </c>
       <c r="Q30" t="n">
-        <v>-0.00554811954498291</v>
+        <v>0.01306992621705083</v>
       </c>
       <c r="R30" t="inlineStr"/>
       <c r="S30" t="inlineStr">
@@ -42784,17 +42784,17 @@
         <v>1</v>
       </c>
       <c r="L32" t="n">
-        <v>26.10000038146973</v>
+        <v>25.8</v>
       </c>
       <c r="M32" t="n">
-        <v>0.4209735095500946</v>
+        <v>0.3637465536594391</v>
       </c>
       <c r="N32" t="n">
-        <v>15.8052978515625</v>
+        <v>27.25068926811218</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>55-60%</t>
+          <t>60-65%</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
@@ -42803,7 +42803,7 @@
         </is>
       </c>
       <c r="Q32" t="n">
-        <v>0.04414272308349609</v>
+        <v>0.1013697254103284</v>
       </c>
       <c r="R32" t="inlineStr"/>
       <c r="S32" t="inlineStr">
@@ -42861,26 +42861,26 @@
         <v>1</v>
       </c>
       <c r="L33" t="n">
-        <v>26.20000076293945</v>
+        <v>25.9</v>
       </c>
       <c r="M33" t="n">
-        <v>0.440240204334259</v>
+        <v>0.3821225464344025</v>
       </c>
       <c r="N33" t="n">
-        <v>11.95195960998535</v>
+        <v>23.57549071311951</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>55-60%</t>
+          <t>60-65%</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>NO BET</t>
+          <t>UNDER</t>
         </is>
       </c>
       <c r="Q33" t="n">
-        <v>0.06956371665000916</v>
+        <v>0.127681375134225</v>
       </c>
       <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr">
@@ -42938,17 +42938,17 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>22.89999961853027</v>
+        <v>22.6</v>
       </c>
       <c r="M34" t="n">
-        <v>0.3793360888957977</v>
+        <v>0.3245962858200073</v>
       </c>
       <c r="N34" t="n">
-        <v>24.13278198242188</v>
+        <v>35.08074283599854</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>60-65%</t>
+          <t>65-70%</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
@@ -42957,7 +42957,7 @@
         </is>
       </c>
       <c r="Q34" t="n">
-        <v>0.06119251251220703</v>
+        <v>0.1159323485412261</v>
       </c>
       <c r="R34" t="inlineStr"/>
       <c r="S34" t="inlineStr">
@@ -43015,17 +43015,17 @@
         <v>1</v>
       </c>
       <c r="L35" t="n">
-        <v>25</v>
+        <v>24.7</v>
       </c>
       <c r="M35" t="n">
-        <v>0.5966944694519043</v>
+        <v>0.5377652049064636</v>
       </c>
       <c r="N35" t="n">
-        <v>19.33889389038086</v>
+        <v>7.553040981292725</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>55-60%</t>
+          <t>50-55%</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
@@ -43034,7 +43034,7 @@
         </is>
       </c>
       <c r="Q35" t="n">
-        <v>0.03722310066223145</v>
+        <v>-0.02170616073230291</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr">
@@ -43092,13 +43092,13 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>23.60000038146973</v>
+        <v>23.3</v>
       </c>
       <c r="M36" t="n">
-        <v>0.5223590135574341</v>
+        <v>0.4623549282550812</v>
       </c>
       <c r="N36" t="n">
-        <v>4.471802711486816</v>
+        <v>7.529014348983765</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
@@ -43111,7 +43111,7 @@
         </is>
       </c>
       <c r="Q36" t="n">
-        <v>0.01255506277084351</v>
+        <v>-0.003639331924805922</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr">
@@ -43169,17 +43169,17 @@
         <v>1</v>
       </c>
       <c r="L37" t="n">
-        <v>26.60000038146973</v>
+        <v>26.4</v>
       </c>
       <c r="M37" t="n">
-        <v>0.7234598398208618</v>
+        <v>0.6728992462158203</v>
       </c>
       <c r="N37" t="n">
-        <v>44.69196701049805</v>
+        <v>34.57984924316406</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>70-75%</t>
+          <t>65-70%</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
@@ -43188,7 +43188,7 @@
         </is>
       </c>
       <c r="Q37" t="n">
-        <v>0.2234598398208618</v>
+        <v>0.1728992462158203</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr">
@@ -43246,13 +43246,13 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>24.70000076293945</v>
+        <v>24.4</v>
       </c>
       <c r="M38" t="n">
-        <v>0.5358247756958008</v>
+        <v>0.4758148491382599</v>
       </c>
       <c r="N38" t="n">
-        <v>7.164955139160156</v>
+        <v>4.837030172348022</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
@@ -43265,7 +43265,7 @@
         </is>
       </c>
       <c r="Q38" t="n">
-        <v>0.04562869668006897</v>
+        <v>-0.01438122929311264</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr">
@@ -43323,26 +43323,26 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>22.89999961853027</v>
+        <v>22.6</v>
       </c>
       <c r="M39" t="n">
-        <v>0.3738554716110229</v>
+        <v>0.3194994032382965</v>
       </c>
       <c r="N39" t="n">
-        <v>25.22890472412109</v>
+        <v>36.1001193523407</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>60-65%</t>
+          <t>65-70%</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>NO BET</t>
+          <t>UNDER</t>
         </is>
       </c>
       <c r="Q39" t="n">
-        <v>0.08068996667861938</v>
+        <v>0.1350460513071581</v>
       </c>
       <c r="R39" t="inlineStr"/>
       <c r="S39" t="inlineStr">
@@ -43354,6 +43354,2316 @@
       <c r="U39" t="inlineStr"/>
       <c r="V39" t="inlineStr"/>
       <c r="W39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>2025021121</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Dobes</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="F40" t="n">
+        <v>-127</v>
+      </c>
+      <c r="G40" t="n">
+        <v>104</v>
+      </c>
+      <c r="H40" t="n">
+        <v>8482487</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>MTL</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>CAR</t>
+        </is>
+      </c>
+      <c r="K40" t="n">
+        <v>1</v>
+      </c>
+      <c r="L40" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="M40" t="n">
+        <v>0.3821225464344025</v>
+      </c>
+      <c r="N40" t="n">
+        <v>23.57549071311951</v>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>60-65%</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>UNDER</t>
+        </is>
+      </c>
+      <c r="Q40" t="n">
+        <v>0.127681375134225</v>
+      </c>
+      <c r="R40" t="inlineStr"/>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr"/>
+      <c r="U40" t="inlineStr"/>
+      <c r="V40" t="inlineStr"/>
+      <c r="W40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>2025021121</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Andersen</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="F41" t="n">
+        <v>102</v>
+      </c>
+      <c r="G41" t="n">
+        <v>-125</v>
+      </c>
+      <c r="H41" t="n">
+        <v>8475883</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>CAR</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>MTL</t>
+        </is>
+      </c>
+      <c r="K41" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" t="n">
+        <v>23</v>
+      </c>
+      <c r="M41" t="n">
+        <v>0.595471203327179</v>
+      </c>
+      <c r="N41" t="n">
+        <v>19.09424066543579</v>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>55-60%</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q41" t="n">
+        <v>0.1004216983766839</v>
+      </c>
+      <c r="R41" t="inlineStr"/>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr"/>
+      <c r="U41" t="inlineStr"/>
+      <c r="V41" t="inlineStr"/>
+      <c r="W41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>2025021126</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Wedgewood</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F42" t="n">
+        <v>-122</v>
+      </c>
+      <c r="G42" t="n">
+        <v>100</v>
+      </c>
+      <c r="H42" t="n">
+        <v>8475809</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>PIT</t>
+        </is>
+      </c>
+      <c r="K42" t="n">
+        <v>0</v>
+      </c>
+      <c r="L42" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="M42" t="n">
+        <v>0.3698245584964752</v>
+      </c>
+      <c r="N42" t="n">
+        <v>26.03508830070496</v>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>60-65%</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>UNDER</t>
+        </is>
+      </c>
+      <c r="Q42" t="n">
+        <v>0.1301754415035248</v>
+      </c>
+      <c r="R42" t="inlineStr"/>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr"/>
+      <c r="U42" t="inlineStr"/>
+      <c r="V42" t="inlineStr"/>
+      <c r="W42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>2025021126</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Silovs</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="F43" t="n">
+        <v>-109</v>
+      </c>
+      <c r="G43" t="n">
+        <v>-113</v>
+      </c>
+      <c r="H43" t="n">
+        <v>8481668</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>PIT</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="K43" t="n">
+        <v>1</v>
+      </c>
+      <c r="L43" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="M43" t="n">
+        <v>0.4212331175804138</v>
+      </c>
+      <c r="N43" t="n">
+        <v>15.75337648391724</v>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>55-60%</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q43" t="n">
+        <v>0.04825045049470356</v>
+      </c>
+      <c r="R43" t="inlineStr"/>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr"/>
+      <c r="U43" t="inlineStr"/>
+      <c r="V43" t="inlineStr"/>
+      <c r="W43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>2025021122</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Ullmark</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F44" t="n">
+        <v>103</v>
+      </c>
+      <c r="G44" t="n">
+        <v>-127</v>
+      </c>
+      <c r="H44" t="n">
+        <v>8476999</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>OTT</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>DET</t>
+        </is>
+      </c>
+      <c r="K44" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="M44" t="n">
+        <v>0.3245962858200073</v>
+      </c>
+      <c r="N44" t="n">
+        <v>35.08074283599854</v>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>65-70%</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q44" t="n">
+        <v>0.1159323485412261</v>
+      </c>
+      <c r="R44" t="inlineStr"/>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr"/>
+      <c r="U44" t="inlineStr"/>
+      <c r="V44" t="inlineStr"/>
+      <c r="W44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>2025021122</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Gibson</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="F45" t="n">
+        <v>-112</v>
+      </c>
+      <c r="G45" t="n">
+        <v>-110</v>
+      </c>
+      <c r="H45" t="n">
+        <v>8476434</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>DET</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>OTT</t>
+        </is>
+      </c>
+      <c r="K45" t="n">
+        <v>1</v>
+      </c>
+      <c r="L45" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="M45" t="n">
+        <v>0.3285265266895294</v>
+      </c>
+      <c r="N45" t="n">
+        <v>34.29469466209412</v>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>65-70%</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>UNDER</t>
+        </is>
+      </c>
+      <c r="Q45" t="n">
+        <v>0.1476639495009467</v>
+      </c>
+      <c r="R45" t="inlineStr"/>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr"/>
+      <c r="U45" t="inlineStr"/>
+      <c r="V45" t="inlineStr"/>
+      <c r="W45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>2025021123</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Daccord</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="F46" t="n">
+        <v>-124</v>
+      </c>
+      <c r="G46" t="n">
+        <v>101</v>
+      </c>
+      <c r="H46" t="n">
+        <v>8478916</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>FLA</t>
+        </is>
+      </c>
+      <c r="K46" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="M46" t="n">
+        <v>0.5223939418792725</v>
+      </c>
+      <c r="N46" t="n">
+        <v>4.478788375854492</v>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>50-55%</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q46" t="n">
+        <v>-0.01990637969021775</v>
+      </c>
+      <c r="R46" t="inlineStr"/>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr"/>
+      <c r="U46" t="inlineStr"/>
+      <c r="V46" t="inlineStr"/>
+      <c r="W46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>2025021123</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Bobrovsky</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="F47" t="n">
+        <v>-112</v>
+      </c>
+      <c r="G47" t="n">
+        <v>-110</v>
+      </c>
+      <c r="H47" t="n">
+        <v>8475683</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>FLA</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="K47" t="n">
+        <v>1</v>
+      </c>
+      <c r="L47" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="M47" t="n">
+        <v>0.6140996217727661</v>
+      </c>
+      <c r="N47" t="n">
+        <v>22.81992435455322</v>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>60-65%</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q47" t="n">
+        <v>0.08579773498031329</v>
+      </c>
+      <c r="R47" t="inlineStr"/>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr"/>
+      <c r="U47" t="inlineStr"/>
+      <c r="V47" t="inlineStr"/>
+      <c r="W47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>2025021125</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Greaves</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F48" t="n">
+        <v>107</v>
+      </c>
+      <c r="G48" t="n">
+        <v>-130</v>
+      </c>
+      <c r="H48" t="n">
+        <v>8482982</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>CBJ</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="K48" t="n">
+        <v>0</v>
+      </c>
+      <c r="L48" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="M48" t="n">
+        <v>0.6457219123840332</v>
+      </c>
+      <c r="N48" t="n">
+        <v>29.14438247680664</v>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>60-65%</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>OVER</t>
+        </is>
+      </c>
+      <c r="Q48" t="n">
+        <v>0.1626301249444197</v>
+      </c>
+      <c r="R48" t="inlineStr"/>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr"/>
+      <c r="U48" t="inlineStr"/>
+      <c r="V48" t="inlineStr"/>
+      <c r="W48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>2025021125</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Vladar</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="F49" t="n">
+        <v>-107</v>
+      </c>
+      <c r="G49" t="n">
+        <v>-115</v>
+      </c>
+      <c r="H49" t="n">
+        <v>8478435</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>CBJ</t>
+        </is>
+      </c>
+      <c r="K49" t="n">
+        <v>1</v>
+      </c>
+      <c r="L49" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="M49" t="n">
+        <v>0.6251416206359863</v>
+      </c>
+      <c r="N49" t="n">
+        <v>25.02832412719727</v>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>60-65%</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q49" t="n">
+        <v>0.1082334080755999</v>
+      </c>
+      <c r="R49" t="inlineStr"/>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr"/>
+      <c r="U49" t="inlineStr"/>
+      <c r="V49" t="inlineStr"/>
+      <c r="W49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>2025021124</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Soderblom</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="F50" t="n">
+        <v>-108</v>
+      </c>
+      <c r="G50" t="n">
+        <v>-114</v>
+      </c>
+      <c r="H50" t="n">
+        <v>8482821</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>CHI</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>NYI</t>
+        </is>
+      </c>
+      <c r="K50" t="n">
+        <v>0</v>
+      </c>
+      <c r="L50" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="M50" t="n">
+        <v>0.3604073524475098</v>
+      </c>
+      <c r="N50" t="n">
+        <v>27.91852951049805</v>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>60-65%</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q50" t="n">
+        <v>0.1068823671786585</v>
+      </c>
+      <c r="R50" t="inlineStr"/>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr"/>
+      <c r="U50" t="inlineStr"/>
+      <c r="V50" t="inlineStr"/>
+      <c r="W50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>2025021124</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Rittich</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="F51" t="n">
+        <v>-108</v>
+      </c>
+      <c r="G51" t="n">
+        <v>-114</v>
+      </c>
+      <c r="H51" t="n">
+        <v>8479496</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>NYI</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>CHI</t>
+        </is>
+      </c>
+      <c r="K51" t="n">
+        <v>1</v>
+      </c>
+      <c r="L51" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="M51" t="n">
+        <v>0.579328715801239</v>
+      </c>
+      <c r="N51" t="n">
+        <v>15.8657431602478</v>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>55-60%</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q51" t="n">
+        <v>0.06009794657046974</v>
+      </c>
+      <c r="R51" t="inlineStr"/>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr"/>
+      <c r="U51" t="inlineStr"/>
+      <c r="V51" t="inlineStr"/>
+      <c r="W51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>2025021120</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Stolarz</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="F52" t="n">
+        <v>-106</v>
+      </c>
+      <c r="G52" t="n">
+        <v>-117</v>
+      </c>
+      <c r="H52" t="n">
+        <v>8476932</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>BOS</t>
+        </is>
+      </c>
+      <c r="K52" t="n">
+        <v>0</v>
+      </c>
+      <c r="L52" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="M52" t="n">
+        <v>0.4775381088256836</v>
+      </c>
+      <c r="N52" t="n">
+        <v>4.492378234863281</v>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>50-55%</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q52" t="n">
+        <v>-0.01670861573812599</v>
+      </c>
+      <c r="R52" t="inlineStr"/>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr"/>
+      <c r="U52" t="inlineStr"/>
+      <c r="V52" t="inlineStr"/>
+      <c r="W52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>2025021120</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Swayman</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F53" t="n">
+        <v>-110</v>
+      </c>
+      <c r="G53" t="n">
+        <v>-112</v>
+      </c>
+      <c r="H53" t="n">
+        <v>8480280</v>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>BOS</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="K53" t="n">
+        <v>1</v>
+      </c>
+      <c r="L53" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="M53" t="n">
+        <v>0.4317587614059448</v>
+      </c>
+      <c r="N53" t="n">
+        <v>13.64824771881104</v>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>55-60%</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q53" t="n">
+        <v>0.03993935180160235</v>
+      </c>
+      <c r="R53" t="inlineStr"/>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr"/>
+      <c r="U53" t="inlineStr"/>
+      <c r="V53" t="inlineStr"/>
+      <c r="W53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>2025021127</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Gustavsson</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="F54" t="n">
+        <v>101</v>
+      </c>
+      <c r="G54" t="n">
+        <v>-124</v>
+      </c>
+      <c r="H54" t="n">
+        <v>8479406</v>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>MIN</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>TBL</t>
+        </is>
+      </c>
+      <c r="K54" t="n">
+        <v>0</v>
+      </c>
+      <c r="L54" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="M54" t="n">
+        <v>0.2300351709127426</v>
+      </c>
+      <c r="N54" t="n">
+        <v>53.99296581745148</v>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>75%+</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>UNDER</t>
+        </is>
+      </c>
+      <c r="Q54" t="n">
+        <v>0.2163934005158288</v>
+      </c>
+      <c r="R54" t="inlineStr"/>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr"/>
+      <c r="U54" t="inlineStr"/>
+      <c r="V54" t="inlineStr"/>
+      <c r="W54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>2025021127</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Vasilevskiy</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="F55" t="n">
+        <v>-127</v>
+      </c>
+      <c r="G55" t="n">
+        <v>104</v>
+      </c>
+      <c r="H55" t="n">
+        <v>8476883</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>TBL</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>MIN</t>
+        </is>
+      </c>
+      <c r="K55" t="n">
+        <v>1</v>
+      </c>
+      <c r="L55" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="M55" t="n">
+        <v>0.5377652049064636</v>
+      </c>
+      <c r="N55" t="n">
+        <v>7.553040981292725</v>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>50-55%</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q55" t="n">
+        <v>-0.02170616073230291</v>
+      </c>
+      <c r="R55" t="inlineStr"/>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr"/>
+      <c r="U55" t="inlineStr"/>
+      <c r="V55" t="inlineStr"/>
+      <c r="W55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>2025021130</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Allen</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F56" t="n">
+        <v>-104</v>
+      </c>
+      <c r="G56" t="n">
+        <v>-118</v>
+      </c>
+      <c r="H56" t="n">
+        <v>8474596</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>NJD</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="K56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L56" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="M56" t="n">
+        <v>0.4623549282550812</v>
+      </c>
+      <c r="N56" t="n">
+        <v>7.529014348983765</v>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>50-55%</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q56" t="n">
+        <v>-0.003639331924805922</v>
+      </c>
+      <c r="R56" t="inlineStr"/>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T56" t="inlineStr"/>
+      <c r="U56" t="inlineStr"/>
+      <c r="V56" t="inlineStr"/>
+      <c r="W56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>2025021130</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Oettinger</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="F57" t="n">
+        <v>100</v>
+      </c>
+      <c r="G57" t="n">
+        <v>-122</v>
+      </c>
+      <c r="H57" t="n">
+        <v>8479979</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>NJD</t>
+        </is>
+      </c>
+      <c r="K57" t="n">
+        <v>1</v>
+      </c>
+      <c r="L57" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="M57" t="n">
+        <v>0.2381392866373062</v>
+      </c>
+      <c r="N57" t="n">
+        <v>52.37214267253876</v>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>75%+</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>UNDER</t>
+        </is>
+      </c>
+      <c r="Q57" t="n">
+        <v>0.2123111638131442</v>
+      </c>
+      <c r="R57" t="inlineStr"/>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr"/>
+      <c r="U57" t="inlineStr"/>
+      <c r="V57" t="inlineStr"/>
+      <c r="W57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>2025021129</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Saros</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="F58" t="n">
+        <v>-106</v>
+      </c>
+      <c r="G58" t="n">
+        <v>-117</v>
+      </c>
+      <c r="H58" t="n">
+        <v>8477424</v>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>NSH</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>SJS</t>
+        </is>
+      </c>
+      <c r="K58" t="n">
+        <v>1</v>
+      </c>
+      <c r="L58" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="M58" t="n">
+        <v>0.4699823558330536</v>
+      </c>
+      <c r="N58" t="n">
+        <v>6.003528833389282</v>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>50-55%</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q58" t="n">
+        <v>-0.009152862745495982</v>
+      </c>
+      <c r="R58" t="inlineStr"/>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T58" t="inlineStr"/>
+      <c r="U58" t="inlineStr"/>
+      <c r="V58" t="inlineStr"/>
+      <c r="W58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>2025021129</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Nedeljkovic</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="F59" t="n">
+        <v>-107</v>
+      </c>
+      <c r="G59" t="n">
+        <v>-115</v>
+      </c>
+      <c r="H59" t="n">
+        <v>8477968</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>SJS</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>NSH</t>
+        </is>
+      </c>
+      <c r="K59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L59" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="M59" t="n">
+        <v>0.4220030903816223</v>
+      </c>
+      <c r="N59" t="n">
+        <v>15.59938192367554</v>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>55-60%</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q59" t="n">
+        <v>0.04311318868814518</v>
+      </c>
+      <c r="R59" t="inlineStr"/>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr"/>
+      <c r="U59" t="inlineStr"/>
+      <c r="V59" t="inlineStr"/>
+      <c r="W59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>2025021131</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Hill</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="F60" t="n">
+        <v>-109</v>
+      </c>
+      <c r="G60" t="n">
+        <v>-113</v>
+      </c>
+      <c r="H60" t="n">
+        <v>8478499</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>VGK</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>WPG</t>
+        </is>
+      </c>
+      <c r="K60" t="n">
+        <v>0</v>
+      </c>
+      <c r="L60" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="M60" t="n">
+        <v>0.5564432144165039</v>
+      </c>
+      <c r="N60" t="n">
+        <v>11.28864288330078</v>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>55-60%</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q60" t="n">
+        <v>0.03491211393803506</v>
+      </c>
+      <c r="R60" t="inlineStr"/>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr"/>
+      <c r="U60" t="inlineStr"/>
+      <c r="V60" t="inlineStr"/>
+      <c r="W60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>2025021131</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Hellebuyck</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="F61" t="n">
+        <v>100</v>
+      </c>
+      <c r="G61" t="n">
+        <v>-122</v>
+      </c>
+      <c r="H61" t="n">
+        <v>8476945</v>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>WPG</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>VGK</t>
+        </is>
+      </c>
+      <c r="K61" t="n">
+        <v>1</v>
+      </c>
+      <c r="L61" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="M61" t="n">
+        <v>0.6728992462158203</v>
+      </c>
+      <c r="N61" t="n">
+        <v>34.57984924316406</v>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>65-70%</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>OVER</t>
+        </is>
+      </c>
+      <c r="Q61" t="n">
+        <v>0.1728992462158203</v>
+      </c>
+      <c r="R61" t="inlineStr"/>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T61" t="inlineStr"/>
+      <c r="U61" t="inlineStr"/>
+      <c r="V61" t="inlineStr"/>
+      <c r="W61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>2025021128</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Hofer</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="F62" t="n">
+        <v>-107</v>
+      </c>
+      <c r="G62" t="n">
+        <v>-114</v>
+      </c>
+      <c r="H62" t="n">
+        <v>8480981</v>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>WSH</t>
+        </is>
+      </c>
+      <c r="K62" t="n">
+        <v>1</v>
+      </c>
+      <c r="L62" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="M62" t="n">
+        <v>0.4552974998950958</v>
+      </c>
+      <c r="N62" t="n">
+        <v>8.940500020980835</v>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>50-55%</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q62" t="n">
+        <v>0.01199221973107245</v>
+      </c>
+      <c r="R62" t="inlineStr"/>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T62" t="inlineStr"/>
+      <c r="U62" t="inlineStr"/>
+      <c r="V62" t="inlineStr"/>
+      <c r="W62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>2025021128</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Lindgren</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F63" t="n">
+        <v>100</v>
+      </c>
+      <c r="G63" t="n">
+        <v>-124</v>
+      </c>
+      <c r="H63" t="n">
+        <v>8479292</v>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>WSH</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="K63" t="n">
+        <v>0</v>
+      </c>
+      <c r="L63" t="n">
+        <v>23</v>
+      </c>
+      <c r="M63" t="n">
+        <v>0.409813404083252</v>
+      </c>
+      <c r="N63" t="n">
+        <v>18.03731918334961</v>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>55-60%</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q63" t="n">
+        <v>0.03661516734531944</v>
+      </c>
+      <c r="R63" t="inlineStr"/>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr"/>
+      <c r="U63" t="inlineStr"/>
+      <c r="V63" t="inlineStr"/>
+      <c r="W63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>2025021133</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Wolf</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="F64" t="n">
+        <v>-103</v>
+      </c>
+      <c r="G64" t="n">
+        <v>-120</v>
+      </c>
+      <c r="H64" t="n">
+        <v>8481692</v>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>CGY</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>LAK</t>
+        </is>
+      </c>
+      <c r="K64" t="n">
+        <v>1</v>
+      </c>
+      <c r="L64" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="M64" t="n">
+        <v>0.3082170188426971</v>
+      </c>
+      <c r="N64" t="n">
+        <v>38.35659623146057</v>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>65-70%</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>UNDER</t>
+        </is>
+      </c>
+      <c r="Q64" t="n">
+        <v>0.1463284357027574</v>
+      </c>
+      <c r="R64" t="inlineStr"/>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T64" t="inlineStr"/>
+      <c r="U64" t="inlineStr"/>
+      <c r="V64" t="inlineStr"/>
+      <c r="W64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>2025021133</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Kuemper</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F65" t="n">
+        <v>-121</v>
+      </c>
+      <c r="G65" t="n">
+        <v>-102</v>
+      </c>
+      <c r="H65" t="n">
+        <v>8475311</v>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>LAK</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>CGY</t>
+        </is>
+      </c>
+      <c r="K65" t="n">
+        <v>0</v>
+      </c>
+      <c r="L65" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="M65" t="n">
+        <v>0.4819795787334442</v>
+      </c>
+      <c r="N65" t="n">
+        <v>3.604084253311157</v>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>50-55%</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q65" t="n">
+        <v>0.01306992621705083</v>
+      </c>
+      <c r="R65" t="inlineStr"/>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr"/>
+      <c r="U65" t="inlineStr"/>
+      <c r="V65" t="inlineStr"/>
+      <c r="W65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>2025021132</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Jarry</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="F66" t="n">
+        <v>104</v>
+      </c>
+      <c r="G66" t="n">
+        <v>-127</v>
+      </c>
+      <c r="H66" t="n">
+        <v>8477465</v>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>EDM</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>UTA</t>
+        </is>
+      </c>
+      <c r="K66" t="n">
+        <v>0</v>
+      </c>
+      <c r="L66" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="M66" t="n">
+        <v>0.4758148491382599</v>
+      </c>
+      <c r="N66" t="n">
+        <v>4.837030172348022</v>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>50-55%</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q66" t="n">
+        <v>-0.01438122929311264</v>
+      </c>
+      <c r="R66" t="inlineStr"/>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T66" t="inlineStr"/>
+      <c r="U66" t="inlineStr"/>
+      <c r="V66" t="inlineStr"/>
+      <c r="W66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>2025021132</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Vejmelka</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="F67" t="n">
+        <v>101</v>
+      </c>
+      <c r="G67" t="n">
+        <v>-124</v>
+      </c>
+      <c r="H67" t="n">
+        <v>8478872</v>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>UTA</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>EDM</t>
+        </is>
+      </c>
+      <c r="K67" t="n">
+        <v>1</v>
+      </c>
+      <c r="L67" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="M67" t="n">
+        <v>0.6984090805053711</v>
+      </c>
+      <c r="N67" t="n">
+        <v>39.68181610107422</v>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>65-70%</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>OVER</t>
+        </is>
+      </c>
+      <c r="Q67" t="n">
+        <v>0.2008966426944258</v>
+      </c>
+      <c r="R67" t="inlineStr"/>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T67" t="inlineStr"/>
+      <c r="U67" t="inlineStr"/>
+      <c r="V67" t="inlineStr"/>
+      <c r="W67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>2025021134</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Dostal</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F68" t="n">
+        <v>-104</v>
+      </c>
+      <c r="G68" t="n">
+        <v>-120</v>
+      </c>
+      <c r="H68" t="n">
+        <v>8480843</v>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>ANA</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>VAN</t>
+        </is>
+      </c>
+      <c r="K68" t="n">
+        <v>0</v>
+      </c>
+      <c r="L68" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="M68" t="n">
+        <v>0.3194994032382965</v>
+      </c>
+      <c r="N68" t="n">
+        <v>36.1001193523407</v>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>65-70%</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>UNDER</t>
+        </is>
+      </c>
+      <c r="Q68" t="n">
+        <v>0.1350460513071581</v>
+      </c>
+      <c r="R68" t="inlineStr"/>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T68" t="inlineStr"/>
+      <c r="U68" t="inlineStr"/>
+      <c r="V68" t="inlineStr"/>
+      <c r="W68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>2025021134</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Lankinen</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="F69" t="n">
+        <v>-107</v>
+      </c>
+      <c r="G69" t="n">
+        <v>-115</v>
+      </c>
+      <c r="H69" t="n">
+        <v>8480947</v>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>VAN</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>ANA</t>
+        </is>
+      </c>
+      <c r="K69" t="n">
+        <v>1</v>
+      </c>
+      <c r="L69" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="M69" t="n">
+        <v>0.3637465536594391</v>
+      </c>
+      <c r="N69" t="n">
+        <v>27.25068926811218</v>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>60-65%</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q69" t="n">
+        <v>0.1013697254103284</v>
+      </c>
+      <c r="R69" t="inlineStr"/>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T69" t="inlineStr"/>
+      <c r="U69" t="inlineStr"/>
+      <c r="V69" t="inlineStr"/>
+      <c r="W69" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update betting results for 2026-03-27
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -38222,9 +38222,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
+      <c r="T2" t="n">
+        <v>28</v>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V2" t="n">
+        <v>0</v>
+      </c>
       <c r="W2" t="inlineStr"/>
     </row>
     <row r="3">
@@ -38299,9 +38307,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
+      <c r="T3" t="n">
+        <v>15</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V3" t="n">
+        <v>0</v>
+      </c>
       <c r="W3" t="inlineStr"/>
     </row>
     <row r="4">
@@ -38376,9 +38392,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
+      <c r="T4" t="n">
+        <v>33</v>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V4" t="n">
+        <v>0</v>
+      </c>
       <c r="W4" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update betting results for 2026-03-27 (#29)
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -38222,9 +38222,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
+      <c r="T2" t="n">
+        <v>28</v>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V2" t="n">
+        <v>0</v>
+      </c>
       <c r="W2" t="inlineStr"/>
     </row>
     <row r="3">
@@ -38299,9 +38307,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
+      <c r="T3" t="n">
+        <v>15</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V3" t="n">
+        <v>0</v>
+      </c>
       <c r="W3" t="inlineStr"/>
     </row>
     <row r="4">
@@ -38376,9 +38392,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
+      <c r="T4" t="n">
+        <v>33</v>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V4" t="n">
+        <v>0</v>
+      </c>
       <c r="W4" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update betting_tracker with latest predictions (#32)
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -37898,7 +37898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W6"/>
+  <dimension ref="A1:W13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38402,6 +38402,545 @@
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2025021163</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Vladar</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-106</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-117</v>
+      </c>
+      <c r="H7" t="n">
+        <v>8478435</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>DET</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>24.29999923706055</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.4616363346576691</v>
+      </c>
+      <c r="N7" t="n">
+        <v>7.672733306884766</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>50-55%</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q7" t="n">
+        <v>-0.0008068084716796875</v>
+      </c>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2025021165</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Wolf</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-107</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-115</v>
+      </c>
+      <c r="H8" t="n">
+        <v>8481692</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>CGY</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>VAN</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" t="n">
+        <v>23.10000038146973</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.4227294623851776</v>
+      </c>
+      <c r="N8" t="n">
+        <v>15.4541072845459</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>55-60%</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
+        <v>0.04238677024841309</v>
+      </c>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2025021161</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Fowler</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-121</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-102</v>
+      </c>
+      <c r="H9" t="n">
+        <v>8484170</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>MTL</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>NSH</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>22.70000076293945</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.3324140608310699</v>
+      </c>
+      <c r="N9" t="n">
+        <v>33.51718902587891</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>65-70%</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>UNDER</t>
+        </is>
+      </c>
+      <c r="Q9" t="n">
+        <v>0.1626354455947876</v>
+      </c>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2025021160</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Woll</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-125</v>
+      </c>
+      <c r="G10" t="n">
+        <v>102</v>
+      </c>
+      <c r="H10" t="n">
+        <v>8479361</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>25</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.4005590081214905</v>
+      </c>
+      <c r="N10" t="n">
+        <v>19.88819885253906</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>55-60%</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>0.104391485452652</v>
+      </c>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2025021152</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Reimer</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-121</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-102</v>
+      </c>
+      <c r="H11" t="n">
+        <v>8473503</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>OTT</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>TBL</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>22</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.4008736312389374</v>
+      </c>
+      <c r="N11" t="n">
+        <v>19.82527351379395</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>55-60%</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q11" t="n">
+        <v>0.09417581558227539</v>
+      </c>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>2025021152</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Vasilevskiy</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-103</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-121</v>
+      </c>
+      <c r="H12" t="n">
+        <v>8476883</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>TBL</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>OTT</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>1</v>
+      </c>
+      <c r="L12" t="n">
+        <v>24</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.3939701318740845</v>
+      </c>
+      <c r="N12" t="n">
+        <v>21.20597457885742</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>60-65%</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q12" t="n">
+        <v>0.05851852893829346</v>
+      </c>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2025021153</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Sorokin</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-125</v>
+      </c>
+      <c r="G13" t="n">
+        <v>102</v>
+      </c>
+      <c r="H13" t="n">
+        <v>8478009</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>NYI</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>FLA</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" t="n">
+        <v>22.89999961853027</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.3788540065288544</v>
+      </c>
+      <c r="N13" t="n">
+        <v>24.22919845581055</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>60-65%</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>UNDER</t>
+        </is>
+      </c>
+      <c r="Q13" t="n">
+        <v>0.1260964572429657</v>
+      </c>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr"/>
+      <c r="W13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update betting_tracker with latest predictions (#43)
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -38656,7 +38656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W2"/>
+  <dimension ref="A1:W10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38852,6 +38852,622 @@
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2025021173</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Silovs</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-118</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-105</v>
+      </c>
+      <c r="H3" t="n">
+        <v>8481668</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>PIT</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>NYI</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>23.89999961853027</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.3759295344352722</v>
+      </c>
+      <c r="N3" t="n">
+        <v>24.8140926361084</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>60-65%</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>0.1118753552436829</v>
+      </c>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2025021173</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Sorokin</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-113</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-110</v>
+      </c>
+      <c r="H4" t="n">
+        <v>8478009</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>NYI</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>PIT</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" t="n">
+        <v>23.60000038146973</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.3244228065013885</v>
+      </c>
+      <c r="N4" t="n">
+        <v>35.11544036865234</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>65-70%</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>UNDER</t>
+        </is>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.1517676115036011</v>
+      </c>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2025021174</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Wedgewood</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="F5" t="n">
+        <v>103</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-127</v>
+      </c>
+      <c r="H5" t="n">
+        <v>8475809</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>CGY</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.5070978999137878</v>
+      </c>
+      <c r="N5" t="n">
+        <v>1.419579982757568</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>50-55%</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.01448705792427063</v>
+      </c>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2025021174</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Wolf</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-105</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-118</v>
+      </c>
+      <c r="H6" t="n">
+        <v>8481692</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>CGY</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>28.89999961853027</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.1802056878805161</v>
+      </c>
+      <c r="N6" t="n">
+        <v>63.95885848999023</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>75%+</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>UNDER</t>
+        </is>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.2785099148750305</v>
+      </c>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2025021176</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Husso</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-118</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-105</v>
+      </c>
+      <c r="H7" t="n">
+        <v>8478024</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>ANA</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" t="n">
+        <v>21.89999961853027</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.3868311643600464</v>
+      </c>
+      <c r="N7" t="n">
+        <v>22.63376617431641</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>60-65%</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q7" t="n">
+        <v>0.1009737253189087</v>
+      </c>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2025021176</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Stolarz</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-107</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-115</v>
+      </c>
+      <c r="H8" t="n">
+        <v>8476932</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>ANA</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>29.70000076293945</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.3459508419036865</v>
+      </c>
+      <c r="N8" t="n">
+        <v>30.8098316192627</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>65-70%</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
+        <v>0.1191654205322266</v>
+      </c>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2025021177</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Askarov</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-110</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-112</v>
+      </c>
+      <c r="H9" t="n">
+        <v>8482137</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>SJS</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>1</v>
+      </c>
+      <c r="L9" t="n">
+        <v>23</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.605582594871521</v>
+      </c>
+      <c r="N9" t="n">
+        <v>21.11651992797852</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>60-65%</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q9" t="n">
+        <v>0.08177304267883301</v>
+      </c>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2025021177</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Hofer</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-107</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-115</v>
+      </c>
+      <c r="H10" t="n">
+        <v>8480981</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>SJS</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>24.29999923706055</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.4614397883415222</v>
+      </c>
+      <c r="N10" t="n">
+        <v>7.712042331695557</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>50-55%</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>0.003676474094390869</v>
+      </c>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update betting_tracker with latest predictions (#45)
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -44772,7 +44772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W23"/>
+  <dimension ref="A1:W28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -46599,6 +46599,391 @@
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr"/>
       <c r="W23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>2025021179</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Sorokin</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="F24" t="n">
+        <v>-106</v>
+      </c>
+      <c r="G24" t="n">
+        <v>-117</v>
+      </c>
+      <c r="H24" t="n">
+        <v>8478009</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>NYI</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>BUF</t>
+        </is>
+      </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" t="n">
+        <v>24.10000038146973</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0.2221478819847107</v>
+      </c>
+      <c r="N24" t="n">
+        <v>55.5704231262207</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>75%+</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>UNDER</t>
+        </is>
+      </c>
+      <c r="Q24" t="n">
+        <v>0.2386816143989563</v>
+      </c>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>2025021183</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Gibson</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="F25" t="n">
+        <v>-110</v>
+      </c>
+      <c r="G25" t="n">
+        <v>-112</v>
+      </c>
+      <c r="H25" t="n">
+        <v>8476434</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>DET</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>PIT</t>
+        </is>
+      </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" t="n">
+        <v>24.29999923706055</v>
+      </c>
+      <c r="M25" t="n">
+        <v>0.258517324924469</v>
+      </c>
+      <c r="N25" t="n">
+        <v>48.29653549194336</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>70-75%</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>UNDER</t>
+        </is>
+      </c>
+      <c r="Q25" t="n">
+        <v>0.2131807804107666</v>
+      </c>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr"/>
+      <c r="W25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>2025021181</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Ullmark</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="F26" t="n">
+        <v>-121</v>
+      </c>
+      <c r="G26" t="n">
+        <v>-103</v>
+      </c>
+      <c r="H26" t="n">
+        <v>8476999</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>OTT</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>FLA</t>
+        </is>
+      </c>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" t="n">
+        <v>22.29999923706055</v>
+      </c>
+      <c r="M26" t="n">
+        <v>0.4507530033588409</v>
+      </c>
+      <c r="N26" t="n">
+        <v>9.849399566650391</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>50-55%</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q26" t="n">
+        <v>0.04185783863067627</v>
+      </c>
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr"/>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="inlineStr"/>
+      <c r="W26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>2025021186</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Knight</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="F27" t="n">
+        <v>102</v>
+      </c>
+      <c r="G27" t="n">
+        <v>-125</v>
+      </c>
+      <c r="H27" t="n">
+        <v>8481519</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>CHI</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>WPG</t>
+        </is>
+      </c>
+      <c r="K27" t="n">
+        <v>1</v>
+      </c>
+      <c r="L27" t="n">
+        <v>24.60000038146973</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0.3186401426792145</v>
+      </c>
+      <c r="N27" t="n">
+        <v>36.27197265625</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>65-70%</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>UNDER</t>
+        </is>
+      </c>
+      <c r="Q27" t="n">
+        <v>0.1258043050765991</v>
+      </c>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr"/>
+      <c r="W27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>2025021186</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Hellebuyck</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="F28" t="n">
+        <v>-108</v>
+      </c>
+      <c r="G28" t="n">
+        <v>-114</v>
+      </c>
+      <c r="H28" t="n">
+        <v>8476945</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>WPG</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>CHI</t>
+        </is>
+      </c>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" t="n">
+        <v>22.70000076293945</v>
+      </c>
+      <c r="M28" t="n">
+        <v>0.5318290591239929</v>
+      </c>
+      <c r="N28" t="n">
+        <v>6.365811824798584</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>50-55%</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q28" t="n">
+        <v>0.01259827613830566</v>
+      </c>
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr"/>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr"/>
+      <c r="W28" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update betting results for 2026-03-31
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -44964,9 +44964,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
+      <c r="T2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V2" t="n">
+        <v>0</v>
+      </c>
       <c r="W2" t="inlineStr"/>
     </row>
     <row r="3">
@@ -45041,9 +45049,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
+      <c r="T3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V3" t="n">
+        <v>0</v>
+      </c>
       <c r="W3" t="inlineStr"/>
     </row>
     <row r="4">
@@ -45120,9 +45136,17 @@
           <t>OVER</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
+      <c r="T4" t="n">
+        <v>22</v>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="V4" t="n">
+        <v>-2</v>
+      </c>
       <c r="W4" t="inlineStr"/>
     </row>
     <row r="5">
@@ -45199,9 +45223,17 @@
           <t>UNDER</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
+      <c r="T5" t="n">
+        <v>11</v>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="V5" t="n">
+        <v>1.739130434782608</v>
+      </c>
       <c r="W5" t="inlineStr"/>
     </row>
     <row r="6">
@@ -45276,9 +45308,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
+      <c r="T6" t="n">
+        <v>25</v>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V6" t="n">
+        <v>0</v>
+      </c>
       <c r="W6" t="inlineStr"/>
     </row>
     <row r="7">
@@ -45355,9 +45395,17 @@
           <t>OVER</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
+      <c r="T7" t="n">
+        <v>18</v>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="V7" t="n">
+        <v>-1</v>
+      </c>
       <c r="W7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -45432,9 +45480,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
+      <c r="T8" t="n">
+        <v>22</v>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V8" t="n">
+        <v>0</v>
+      </c>
       <c r="W8" t="inlineStr"/>
     </row>
     <row r="9">
@@ -45509,9 +45565,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr"/>
+      <c r="T9" t="n">
+        <v>23</v>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V9" t="n">
+        <v>0</v>
+      </c>
       <c r="W9" t="inlineStr"/>
     </row>
     <row r="10">
@@ -45586,9 +45650,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr"/>
+      <c r="T10" t="n">
+        <v>12</v>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V10" t="n">
+        <v>0</v>
+      </c>
       <c r="W10" t="inlineStr"/>
     </row>
     <row r="11">
@@ -45663,9 +45735,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T11" t="inlineStr"/>
-      <c r="U11" t="inlineStr"/>
-      <c r="V11" t="inlineStr"/>
+      <c r="T11" t="n">
+        <v>17</v>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V11" t="n">
+        <v>0</v>
+      </c>
       <c r="W11" t="inlineStr"/>
     </row>
     <row r="12">
@@ -45742,9 +45822,17 @@
           <t>UNDER</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr"/>
-      <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr"/>
+      <c r="T12" t="n">
+        <v>13</v>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="V12" t="n">
+        <v>1</v>
+      </c>
       <c r="W12" t="inlineStr"/>
     </row>
     <row r="13">
@@ -45819,9 +45907,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T13" t="inlineStr"/>
-      <c r="U13" t="inlineStr"/>
-      <c r="V13" t="inlineStr"/>
+      <c r="T13" t="n">
+        <v>36</v>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V13" t="n">
+        <v>0</v>
+      </c>
       <c r="W13" t="inlineStr"/>
     </row>
     <row r="14">
@@ -45898,9 +45994,17 @@
           <t>UNDER</t>
         </is>
       </c>
-      <c r="T14" t="inlineStr"/>
-      <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr"/>
+      <c r="T14" t="n">
+        <v>19</v>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="V14" t="n">
+        <v>0.9090909090909092</v>
+      </c>
       <c r="W14" t="inlineStr"/>
     </row>
     <row r="15">
@@ -45975,9 +46079,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T15" t="inlineStr"/>
-      <c r="U15" t="inlineStr"/>
-      <c r="V15" t="inlineStr"/>
+      <c r="T15" t="n">
+        <v>22</v>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V15" t="n">
+        <v>0</v>
+      </c>
       <c r="W15" t="inlineStr"/>
     </row>
     <row r="16">
@@ -46052,9 +46164,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr"/>
+      <c r="T16" t="n">
+        <v>11</v>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V16" t="n">
+        <v>0</v>
+      </c>
       <c r="W16" t="inlineStr"/>
     </row>
     <row r="17">
@@ -46129,9 +46249,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr"/>
+      <c r="T17" t="n">
+        <v>20</v>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V17" t="n">
+        <v>0</v>
+      </c>
       <c r="W17" t="inlineStr"/>
     </row>
     <row r="18">
@@ -46208,9 +46336,17 @@
           <t>UNDER</t>
         </is>
       </c>
-      <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr"/>
+      <c r="T18" t="n">
+        <v>26</v>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="V18" t="n">
+        <v>0.9090909090909092</v>
+      </c>
       <c r="W18" t="inlineStr"/>
     </row>
     <row r="19">
@@ -46285,9 +46421,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T19" t="inlineStr"/>
-      <c r="U19" t="inlineStr"/>
-      <c r="V19" t="inlineStr"/>
+      <c r="T19" t="n">
+        <v>23</v>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V19" t="n">
+        <v>0</v>
+      </c>
       <c r="W19" t="inlineStr"/>
     </row>
     <row r="20">
@@ -46364,9 +46508,17 @@
           <t>UNDER</t>
         </is>
       </c>
-      <c r="T20" t="inlineStr"/>
-      <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr"/>
+      <c r="T20" t="n">
+        <v>20</v>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="V20" t="n">
+        <v>0.8064516129032258</v>
+      </c>
       <c r="W20" t="inlineStr"/>
     </row>
     <row r="21">
@@ -46441,9 +46593,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T21" t="inlineStr"/>
-      <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr"/>
+      <c r="T21" t="n">
+        <v>27</v>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V21" t="n">
+        <v>0</v>
+      </c>
       <c r="W21" t="inlineStr"/>
     </row>
     <row r="22">
@@ -46518,9 +46678,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T22" t="inlineStr"/>
-      <c r="U22" t="inlineStr"/>
-      <c r="V22" t="inlineStr"/>
+      <c r="T22" t="n">
+        <v>22</v>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V22" t="n">
+        <v>0</v>
+      </c>
       <c r="W22" t="inlineStr"/>
     </row>
     <row r="23">
@@ -46595,9 +46763,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T23" t="inlineStr"/>
-      <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr"/>
+      <c r="T23" t="n">
+        <v>20</v>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V23" t="n">
+        <v>0</v>
+      </c>
       <c r="W23" t="inlineStr"/>
     </row>
     <row r="24">
@@ -46672,9 +46848,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T24" t="inlineStr"/>
-      <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr"/>
+      <c r="T24" t="n">
+        <v>29</v>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V24" t="n">
+        <v>0</v>
+      </c>
       <c r="W24" t="inlineStr"/>
     </row>
     <row r="25">
@@ -46749,9 +46933,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T25" t="inlineStr"/>
-      <c r="U25" t="inlineStr"/>
-      <c r="V25" t="inlineStr"/>
+      <c r="T25" t="n">
+        <v>11</v>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V25" t="n">
+        <v>0</v>
+      </c>
       <c r="W25" t="inlineStr"/>
     </row>
     <row r="26">
@@ -46826,9 +47018,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T26" t="inlineStr"/>
-      <c r="U26" t="inlineStr"/>
-      <c r="V26" t="inlineStr"/>
+      <c r="T26" t="n">
+        <v>11</v>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V26" t="n">
+        <v>0</v>
+      </c>
       <c r="W26" t="inlineStr"/>
     </row>
     <row r="27">
@@ -46903,9 +47103,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T27" t="inlineStr"/>
-      <c r="U27" t="inlineStr"/>
-      <c r="V27" t="inlineStr"/>
+      <c r="T27" t="n">
+        <v>20</v>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V27" t="n">
+        <v>0</v>
+      </c>
       <c r="W27" t="inlineStr"/>
     </row>
     <row r="28">
@@ -46980,9 +47188,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T28" t="inlineStr"/>
-      <c r="U28" t="inlineStr"/>
-      <c r="V28" t="inlineStr"/>
+      <c r="T28" t="n">
+        <v>18</v>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V28" t="n">
+        <v>0</v>
+      </c>
       <c r="W28" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update betting results for 2026-03-31 (#46)
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -44964,9 +44964,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
+      <c r="T2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V2" t="n">
+        <v>0</v>
+      </c>
       <c r="W2" t="inlineStr"/>
     </row>
     <row r="3">
@@ -45041,9 +45049,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
+      <c r="T3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V3" t="n">
+        <v>0</v>
+      </c>
       <c r="W3" t="inlineStr"/>
     </row>
     <row r="4">
@@ -45120,9 +45136,17 @@
           <t>OVER</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
+      <c r="T4" t="n">
+        <v>22</v>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="V4" t="n">
+        <v>-2</v>
+      </c>
       <c r="W4" t="inlineStr"/>
     </row>
     <row r="5">
@@ -45199,9 +45223,17 @@
           <t>UNDER</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
+      <c r="T5" t="n">
+        <v>11</v>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="V5" t="n">
+        <v>1.739130434782608</v>
+      </c>
       <c r="W5" t="inlineStr"/>
     </row>
     <row r="6">
@@ -45276,9 +45308,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
+      <c r="T6" t="n">
+        <v>25</v>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V6" t="n">
+        <v>0</v>
+      </c>
       <c r="W6" t="inlineStr"/>
     </row>
     <row r="7">
@@ -45355,9 +45395,17 @@
           <t>OVER</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
+      <c r="T7" t="n">
+        <v>18</v>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="V7" t="n">
+        <v>-1</v>
+      </c>
       <c r="W7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -45432,9 +45480,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
+      <c r="T8" t="n">
+        <v>22</v>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V8" t="n">
+        <v>0</v>
+      </c>
       <c r="W8" t="inlineStr"/>
     </row>
     <row r="9">
@@ -45509,9 +45565,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr"/>
+      <c r="T9" t="n">
+        <v>23</v>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V9" t="n">
+        <v>0</v>
+      </c>
       <c r="W9" t="inlineStr"/>
     </row>
     <row r="10">
@@ -45586,9 +45650,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr"/>
+      <c r="T10" t="n">
+        <v>12</v>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V10" t="n">
+        <v>0</v>
+      </c>
       <c r="W10" t="inlineStr"/>
     </row>
     <row r="11">
@@ -45663,9 +45735,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T11" t="inlineStr"/>
-      <c r="U11" t="inlineStr"/>
-      <c r="V11" t="inlineStr"/>
+      <c r="T11" t="n">
+        <v>17</v>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V11" t="n">
+        <v>0</v>
+      </c>
       <c r="W11" t="inlineStr"/>
     </row>
     <row r="12">
@@ -45742,9 +45822,17 @@
           <t>UNDER</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr"/>
-      <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr"/>
+      <c r="T12" t="n">
+        <v>13</v>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="V12" t="n">
+        <v>1</v>
+      </c>
       <c r="W12" t="inlineStr"/>
     </row>
     <row r="13">
@@ -45819,9 +45907,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T13" t="inlineStr"/>
-      <c r="U13" t="inlineStr"/>
-      <c r="V13" t="inlineStr"/>
+      <c r="T13" t="n">
+        <v>36</v>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V13" t="n">
+        <v>0</v>
+      </c>
       <c r="W13" t="inlineStr"/>
     </row>
     <row r="14">
@@ -45898,9 +45994,17 @@
           <t>UNDER</t>
         </is>
       </c>
-      <c r="T14" t="inlineStr"/>
-      <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr"/>
+      <c r="T14" t="n">
+        <v>19</v>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="V14" t="n">
+        <v>0.9090909090909092</v>
+      </c>
       <c r="W14" t="inlineStr"/>
     </row>
     <row r="15">
@@ -45975,9 +46079,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T15" t="inlineStr"/>
-      <c r="U15" t="inlineStr"/>
-      <c r="V15" t="inlineStr"/>
+      <c r="T15" t="n">
+        <v>22</v>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V15" t="n">
+        <v>0</v>
+      </c>
       <c r="W15" t="inlineStr"/>
     </row>
     <row r="16">
@@ -46052,9 +46164,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr"/>
+      <c r="T16" t="n">
+        <v>11</v>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V16" t="n">
+        <v>0</v>
+      </c>
       <c r="W16" t="inlineStr"/>
     </row>
     <row r="17">
@@ -46129,9 +46249,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr"/>
+      <c r="T17" t="n">
+        <v>20</v>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V17" t="n">
+        <v>0</v>
+      </c>
       <c r="W17" t="inlineStr"/>
     </row>
     <row r="18">
@@ -46208,9 +46336,17 @@
           <t>UNDER</t>
         </is>
       </c>
-      <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr"/>
+      <c r="T18" t="n">
+        <v>26</v>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="V18" t="n">
+        <v>0.9090909090909092</v>
+      </c>
       <c r="W18" t="inlineStr"/>
     </row>
     <row r="19">
@@ -46285,9 +46421,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T19" t="inlineStr"/>
-      <c r="U19" t="inlineStr"/>
-      <c r="V19" t="inlineStr"/>
+      <c r="T19" t="n">
+        <v>23</v>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V19" t="n">
+        <v>0</v>
+      </c>
       <c r="W19" t="inlineStr"/>
     </row>
     <row r="20">
@@ -46364,9 +46508,17 @@
           <t>UNDER</t>
         </is>
       </c>
-      <c r="T20" t="inlineStr"/>
-      <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr"/>
+      <c r="T20" t="n">
+        <v>20</v>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="V20" t="n">
+        <v>0.8064516129032258</v>
+      </c>
       <c r="W20" t="inlineStr"/>
     </row>
     <row r="21">
@@ -46441,9 +46593,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T21" t="inlineStr"/>
-      <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr"/>
+      <c r="T21" t="n">
+        <v>27</v>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V21" t="n">
+        <v>0</v>
+      </c>
       <c r="W21" t="inlineStr"/>
     </row>
     <row r="22">
@@ -46518,9 +46678,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T22" t="inlineStr"/>
-      <c r="U22" t="inlineStr"/>
-      <c r="V22" t="inlineStr"/>
+      <c r="T22" t="n">
+        <v>22</v>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V22" t="n">
+        <v>0</v>
+      </c>
       <c r="W22" t="inlineStr"/>
     </row>
     <row r="23">
@@ -46595,9 +46763,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T23" t="inlineStr"/>
-      <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr"/>
+      <c r="T23" t="n">
+        <v>20</v>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V23" t="n">
+        <v>0</v>
+      </c>
       <c r="W23" t="inlineStr"/>
     </row>
     <row r="24">
@@ -46672,9 +46848,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T24" t="inlineStr"/>
-      <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr"/>
+      <c r="T24" t="n">
+        <v>29</v>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V24" t="n">
+        <v>0</v>
+      </c>
       <c r="W24" t="inlineStr"/>
     </row>
     <row r="25">
@@ -46749,9 +46933,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T25" t="inlineStr"/>
-      <c r="U25" t="inlineStr"/>
-      <c r="V25" t="inlineStr"/>
+      <c r="T25" t="n">
+        <v>11</v>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V25" t="n">
+        <v>0</v>
+      </c>
       <c r="W25" t="inlineStr"/>
     </row>
     <row r="26">
@@ -46826,9 +47018,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T26" t="inlineStr"/>
-      <c r="U26" t="inlineStr"/>
-      <c r="V26" t="inlineStr"/>
+      <c r="T26" t="n">
+        <v>11</v>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V26" t="n">
+        <v>0</v>
+      </c>
       <c r="W26" t="inlineStr"/>
     </row>
     <row r="27">
@@ -46903,9 +47103,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T27" t="inlineStr"/>
-      <c r="U27" t="inlineStr"/>
-      <c r="V27" t="inlineStr"/>
+      <c r="T27" t="n">
+        <v>20</v>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V27" t="n">
+        <v>0</v>
+      </c>
       <c r="W27" t="inlineStr"/>
     </row>
     <row r="28">
@@ -46980,9 +47188,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T28" t="inlineStr"/>
-      <c r="U28" t="inlineStr"/>
-      <c r="V28" t="inlineStr"/>
+      <c r="T28" t="n">
+        <v>18</v>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V28" t="n">
+        <v>0</v>
+      </c>
       <c r="W28" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update betting results for 2026-04-03
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -46449,9 +46449,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
+      <c r="T2" t="n">
+        <v>17</v>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V2" t="n">
+        <v>0</v>
+      </c>
       <c r="W2" t="inlineStr"/>
     </row>
     <row r="3">
@@ -46526,9 +46534,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
+      <c r="T3" t="n">
+        <v>21</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V3" t="n">
+        <v>0</v>
+      </c>
       <c r="W3" t="inlineStr"/>
     </row>
     <row r="4">
@@ -46603,9 +46619,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
+      <c r="T4" t="n">
+        <v>23</v>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V4" t="n">
+        <v>0</v>
+      </c>
       <c r="W4" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update betting results for 2026-04-03 (#51)
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -46449,9 +46449,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
+      <c r="T2" t="n">
+        <v>17</v>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V2" t="n">
+        <v>0</v>
+      </c>
       <c r="W2" t="inlineStr"/>
     </row>
     <row r="3">
@@ -46526,9 +46534,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
+      <c r="T3" t="n">
+        <v>21</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V3" t="n">
+        <v>0</v>
+      </c>
       <c r="W3" t="inlineStr"/>
     </row>
     <row r="4">
@@ -46603,9 +46619,17 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
+      <c r="T4" t="n">
+        <v>23</v>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="V4" t="n">
+        <v>0</v>
+      </c>
       <c r="W4" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update betting_tracker with latest predictions (#56)
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -48210,7 +48210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W8"/>
+  <dimension ref="A1:W14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -48868,6 +48868,468 @@
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2025021215</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Hellebuyck</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="F9" t="n">
+        <v>105</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-129</v>
+      </c>
+      <c r="H9" t="n">
+        <v>8476945</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>WPG</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>CBJ</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>24.70000076293945</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.3452522158622742</v>
+      </c>
+      <c r="N9" t="n">
+        <v>30.94955635070801</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>65-70%</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q9" t="n">
+        <v>0.09142899513244629</v>
+      </c>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2025021212</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Allen</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-112</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-110</v>
+      </c>
+      <c r="H10" t="n">
+        <v>8474596</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>NJD</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>MTL</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" t="n">
+        <v>21.79999923706055</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.3623945713043213</v>
+      </c>
+      <c r="N10" t="n">
+        <v>27.52108573913574</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>60-65%</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>0.1137958765029907</v>
+      </c>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2025021220</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Askarov</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-107</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-115</v>
+      </c>
+      <c r="H11" t="n">
+        <v>8482137</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>SJS</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>NSH</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" t="n">
+        <v>24.29999923706055</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.4649761021137238</v>
+      </c>
+      <c r="N11" t="n">
+        <v>7.004779815673828</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>50-55%</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q11" t="n">
+        <v>0.0001401901245117188</v>
+      </c>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>2025021221</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Grubauer</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-102</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-121</v>
+      </c>
+      <c r="H12" t="n">
+        <v>8475831</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>CHI</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>1</v>
+      </c>
+      <c r="L12" t="n">
+        <v>22.89999961853027</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.5878669023513794</v>
+      </c>
+      <c r="N12" t="n">
+        <v>17.57337951660156</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>55-60%</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q12" t="n">
+        <v>0.08291637897491455</v>
+      </c>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2025021218</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Ingram</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-106</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-115</v>
+      </c>
+      <c r="H13" t="n">
+        <v>8478971</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>EDM</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>VGK</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" t="n">
+        <v>23.60000038146973</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.314822643995285</v>
+      </c>
+      <c r="N13" t="n">
+        <v>37.03547286987305</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>65-70%</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>UNDER</t>
+        </is>
+      </c>
+      <c r="Q13" t="n">
+        <v>0.1502935886383057</v>
+      </c>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr"/>
+      <c r="W13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2025021209</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>DeSmith</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-109</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-113</v>
+      </c>
+      <c r="H14" t="n">
+        <v>8479193</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L14" t="n">
+        <v>25.39999961853027</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0.2877406179904938</v>
+      </c>
+      <c r="N14" t="n">
+        <v>42.45187759399414</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>70-75%</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>UNDER</t>
+        </is>
+      </c>
+      <c r="Q14" t="n">
+        <v>0.1817429661750793</v>
+      </c>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update betting_tracker with latest predictions (#69)
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -42308,7 +42308,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W4"/>
+  <dimension ref="A1:W10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -42658,6 +42658,468 @@
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2025021246</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Nedeljkovic</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-104</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-120</v>
+      </c>
+      <c r="H5" t="n">
+        <v>8477968</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>SJS</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>EDM</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" t="n">
+        <v>25</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.4068208336830139</v>
+      </c>
+      <c r="N5" t="n">
+        <v>18.63583374023438</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>55-60%</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.04772460460662842</v>
+      </c>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2025021244</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Luukkonen</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-124</v>
+      </c>
+      <c r="G6" t="n">
+        <v>100</v>
+      </c>
+      <c r="H6" t="n">
+        <v>8480045</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>BUF</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>NYR</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.4973961412906647</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.5207717418670654</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>50-55%</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.002603888511657715</v>
+      </c>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2025021246</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Ingram</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-124</v>
+      </c>
+      <c r="G7" t="n">
+        <v>101</v>
+      </c>
+      <c r="H7" t="n">
+        <v>8478971</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>EDM</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>SJS</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>22.20000076293945</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.4397478401660919</v>
+      </c>
+      <c r="N7" t="n">
+        <v>12.0504322052002</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>55-60%</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q7" t="n">
+        <v>0.06273975968360901</v>
+      </c>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2025021245</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Stolarz</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-127</v>
+      </c>
+      <c r="G8" t="n">
+        <v>104</v>
+      </c>
+      <c r="H8" t="n">
+        <v>8476932</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>WSH</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" t="n">
+        <v>24.79999923706055</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.3542101681232452</v>
+      </c>
+      <c r="N8" t="n">
+        <v>29.15796661376953</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>60-65%</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>UNDER</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
+        <v>0.1555937826633453</v>
+      </c>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2025021244</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Shesterkin</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-127</v>
+      </c>
+      <c r="G9" t="n">
+        <v>104</v>
+      </c>
+      <c r="H9" t="n">
+        <v>8478048</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>NYR</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>BUF</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>1</v>
+      </c>
+      <c r="L9" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.2943671345710754</v>
+      </c>
+      <c r="N9" t="n">
+        <v>41.12657165527344</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>70-75%</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>UNDER</t>
+        </is>
+      </c>
+      <c r="Q9" t="n">
+        <v>0.2154367864131927</v>
+      </c>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2025021245</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Underdog</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Thompson</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-108</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-114</v>
+      </c>
+      <c r="H10" t="n">
+        <v>8480313</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>WSH</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>23</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.3935364186763763</v>
+      </c>
+      <c r="N10" t="n">
+        <v>21.29271697998047</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>60-65%</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>NO BET</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>0.07375329732894897</v>
+      </c>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>